<commit_message>
Fix memory leak and ActiveX COM crash across generations via QuitApplication and _kill_ansys_zombies
</commit_message>
<xml_diff>
--- a/Ai_Optimization_ParamValues.xlsx
+++ b/Ai_Optimization_ParamValues.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,62 +514,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>60</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>23</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>6</v>
-      </c>
-      <c r="M2" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="N2" t="n">
-        <v>4</v>
-      </c>
-      <c r="O2" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>20</v>
-      </c>
-      <c r="R2" t="n">
-        <v>6</v>
-      </c>
-      <c r="S2" t="n">
-        <v>36</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -629,6 +667,200 @@
       </c>
       <c r="S3" t="n">
         <v>48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>